<commit_message>
UI and benchmarks added
</commit_message>
<xml_diff>
--- a/Assets/Data/Rules/Zasady_laczenia_WFC_zamek.xlsx
+++ b/Assets/Data/Rules/Zasady_laczenia_WFC_zamek.xlsx
@@ -29,12 +29,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4027" uniqueCount="743">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4033" uniqueCount="749">
   <si>
     <t xml:space="preserve">Zasady łączenia kostek – WFC zamku</t>
   </si>
   <si>
-    <t xml:space="preserve">Stan na 13.10.2026. W regułach 50 kafelków (170 stanów z obrotami), zestaw ma 48 modeli. Siatka 20 × 20 × 13 kostek po 3 × 3 × 3 m.</t>
+    <t xml:space="preserve">Stan na 21.10.2026. W regułach 50 kafelków (170 stanów z obrotami), zestaw ma 49 modeli. Siatka 20 × 20 × 13 kostek po 3 × 3 × 3 m.</t>
   </si>
   <si>
     <t xml:space="preserve">Zakładki: Kafelki – lista kafelków i etykiet ich ścian · Etykiety – znaczenie każdej etykiety · Zgodność – które etykiety boczne pasują do siebie · Pionowo – co może stać nad czym · Sąsiedzi – pełna lista dozwolonych sąsiadów · Wagi – wagi losowania (można zmieniać) · Poza kostką – elementy wystające poza swoją kostkę · Stany – każdy kafelek w każdym obrocie · Sprawdzenie – wynik testu tych reguł. Wiersze na niebiesko: zasady, które dotąd poprawialiśmy ręcznie, a teraz są w regułach.</t>
@@ -121,7 +121,7 @@
     <t xml:space="preserve">Zakładka Poza kostką</t>
   </si>
   <si>
-    <t xml:space="preserve">Jeden wyjątek do decyzji: filar podestu w Mur_Gora_Przejscie.</t>
+    <t xml:space="preserve">Jeden świadomy wyjątek (decyzja z 21.10.2026): filar podestu w Mur_Gora_Przejscie.</t>
   </si>
   <si>
     <t xml:space="preserve">Teren</t>
@@ -409,7 +409,7 @@
     <t xml:space="preserve">Szczegóły w zakładce Poza kostką.</t>
   </si>
   <si>
-    <t xml:space="preserve">Dach_Szczyt_Choragiew jest w regułach, ale modelu nie ma w zestawie (usunięty z pliku Blendera). Na razie stawiany jest zwykły Dach_Szczyt.</t>
+    <t xml:space="preserve">Dach_Szczyt_Choragiew był w regułach bez modelu: stary model zniknął z pliku Blendera razem ze starym kształtem dachu, więc stawiano zwykły Dach_Szczyt.</t>
   </si>
   <si>
     <t xml:space="preserve">Przywrócić model albo usunąć kafelek.</t>
@@ -883,7 +883,7 @@
     <t xml:space="preserve">Dach_Szczyt_Choragiew</t>
   </si>
   <si>
-    <t xml:space="preserve">Dach_Szczyt_Choragiew (brak w zestawie)</t>
+    <t xml:space="preserve">Dach_Szczyt_Choragiew</t>
   </si>
   <si>
     <t xml:space="preserve">Szczyt dachu z chorągwią.</t>
@@ -1918,7 +1918,7 @@
     <t xml:space="preserve">Pod spodem może stać każdy dół albo środek muru.</t>
   </si>
   <si>
-    <t xml:space="preserve">DO DECYZJI. Koliduje z: Brama_Dol i Brama_Dol_Pochodnie (filar zasłania przejazd), Mur_Dol_Beczki i Mur_Dol_Skrzynie (beczki i skrzynie wchodzą w filar). Bez kolizji: Mur_Dol, Mur_Srodek, Mur_Srodek_V3; Mur_Srodek_V2 – część kamieni chowa się w filarze. W obecnych zamkach jest 6 przejść, pod żadnym nie stoi brama ani dekoracja.</t>
+    <t xml:space="preserve">Świadomy wyjątek (decyzja z 21.10.2026): filar może wchodzić w kostkę muru pod spodem. Koliduje z: Brama_Dol i Brama_Dol_Pochodnie (filar zasłania przejazd), Mur_Dol_Beczki i Mur_Dol_Skrzynie (beczki i skrzynie wchodzą w filar). Bez kolizji: Mur_Dol, Mur_Srodek, Mur_Srodek_V3; Mur_Srodek_V2 – część kamieni chowa się w filarze. W obecnych zamkach jest 6 przejść, pod żadnym nie stoi brama ani dekoracja.</t>
   </si>
   <si>
     <t xml:space="preserve">Pozostałe modele mieszczą się w swojej kostce.</t>
@@ -2258,6 +2258,24 @@
   </si>
   <si>
     <t xml:space="preserve">Poprzednie reguły z brukiem</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozstrzygnięte</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Decyzja z 21.10.2026: świadomy wyjątek, filar może wchodzić w kostkę muru pod spodem. Szczegóły w zakładce Poza kostką.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rozstrzygnięte 21.10.2026: nowy model, czyli kopia Dach_Szczyt z masztem, grotem i proporcem na wierzchołku, wysokość 3,55 m (zakładka Poza kostką).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">w górę: maszt z grotem i proporcem na wierzchołku dachu (proporzec 3,0–3,42 m, grot do 3,55 m nad spodem kostki)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kostka nad</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Nad szczytem dachu zawsze Powietrze. Jeśli na tym Powietrzu stoi most, jego łuk kończy się 0,6 m nad spodem tej kostki, a maszt 0,55 m.</t>
   </si>
 </sst>
 </file>
@@ -2795,7 +2813,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:E70"/>
+  <dimension ref="A1:E71"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -3708,75 +3726,84 @@
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5"/>
       <c r="B66" s="5" t="s">
-        <v>123</v>
+        <v>743</v>
       </c>
       <c r="C66" s="5"/>
       <c r="D66" s="5"/>
       <c r="E66" s="5"/>
     </row>
     <row r="67" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A67" s="10" t="n">
+      <c r="A67" s="6" t="n">
         <v>49</v>
       </c>
-      <c r="B67" s="11" t="s">
+      <c r="B67" s="7" t="s">
+        <v>743</v>
+      </c>
+      <c r="C67" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="D67" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E67" s="7" t="s">
+        <v>744</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A68" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="B68" s="7" t="s">
+        <v>743</v>
+      </c>
+      <c r="C68" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="D68" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="E68" s="7" t="s">
+        <v>745</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A69" s="5"/>
+      <c r="B69" s="5" t="s">
         <v>123</v>
       </c>
-      <c r="C67" s="11" t="s">
-        <v>124</v>
-      </c>
-      <c r="D67" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E67" s="11" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A68" s="10" t="n">
-        <v>50</v>
-      </c>
-      <c r="B68" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="C68" s="11" t="s">
-        <v>126</v>
-      </c>
-      <c r="D68" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E68" s="11" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A69" s="10" t="n">
+      <c r="C69" s="5"/>
+      <c r="D69" s="5"/>
+      <c r="E69" s="5"/>
+    </row>
+    <row r="70" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A70" s="10" t="n">
         <v>51</v>
-      </c>
-      <c r="B69" s="11" t="s">
-        <v>123</v>
-      </c>
-      <c r="C69" s="11" t="s">
-        <v>128</v>
-      </c>
-      <c r="D69" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="E69" s="11"/>
-    </row>
-    <row r="70" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A70" s="10" t="n">
-        <v>52</v>
       </c>
       <c r="B70" s="11" t="s">
         <v>123</v>
       </c>
       <c r="C70" s="11" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="D70" s="11" t="s">
         <v>10</v>
       </c>
-      <c r="E70" s="11" t="s">
+      <c r="E70" s="11"/>
+    </row>
+    <row r="71" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="10" t="n">
+        <v>52</v>
+      </c>
+      <c r="B71" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="C71" s="11" t="s">
+        <v>129</v>
+      </c>
+      <c r="D71" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="E71" s="11" t="s">
         <v>130</v>
       </c>
     </row>
@@ -6530,7 +6557,7 @@
       <c r="B51" s="7" t="s">
         <v>283</v>
       </c>
-      <c r="C51" s="11" t="s">
+      <c r="C51" s="7" t="s">
         <v>284</v>
       </c>
       <c r="D51" s="7" t="s">
@@ -15072,7 +15099,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:F17"/>
+  <dimension ref="A1:F18"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="24"/>
@@ -15314,27 +15341,47 @@
       </c>
     </row>
     <row r="15" customFormat="false" ht="57.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="11" t="s">
+      <c r="A15" s="7" t="s">
         <v>200</v>
       </c>
-      <c r="B15" s="11" t="s">
+      <c r="B15" s="7" t="s">
         <v>626</v>
       </c>
-      <c r="C15" s="25" t="n">
+      <c r="C15" s="23" t="n">
         <v>2.4</v>
       </c>
-      <c r="D15" s="11" t="s">
+      <c r="D15" s="7" t="s">
         <v>627</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="7" t="s">
         <v>628</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="7" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="2" t="s">
+    <row r="16" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="7" t="s">
+        <v>283</v>
+      </c>
+      <c r="B16" s="7" t="s">
+        <v>746</v>
+      </c>
+      <c r="C16" s="23" t="n">
+        <v>0.55</v>
+      </c>
+      <c r="D16" s="7" t="s">
+        <v>747</v>
+      </c>
+      <c r="E16" s="7" t="s">
+        <v>748</v>
+      </c>
+      <c r="F16" s="7" t="s">
+        <v>602</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="2" t="s">
         <v>630</v>
       </c>
     </row>

</xml_diff>